<commit_message>
funciones matematicas medias medianas moda rango
</commit_message>
<xml_diff>
--- a/estadistica-ejercicio-finde/funciones_matematicas.xlsx
+++ b/estadistica-ejercicio-finde/funciones_matematicas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\UsuarioM\Documents\curso_big_data_paula\ejercicio_rombo_y_estadistica_excel\estadistica-ejercicio-finde\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB5BCEFD-9E19-4FB5-9166-64D7D5C24C22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A7414E-21BF-4CD7-86C7-00D9FEB5E94B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="5" xr2:uid="{07B98707-5781-4DBF-A1F8-245D495EAD3C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" firstSheet="4" activeTab="7" xr2:uid="{07B98707-5781-4DBF-A1F8-245D495EAD3C}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -18,12 +18,17 @@
     <sheet name="Hoja3" sheetId="3" r:id="rId3"/>
     <sheet name="MEDIANA" sheetId="4" r:id="rId4"/>
     <sheet name="Monstruo_Choco_Crunch" sheetId="5" r:id="rId5"/>
-    <sheet name="Oferta_Trabajo" sheetId="6" r:id="rId6"/>
+    <sheet name="ejemplo4_tabla_sueldos" sheetId="6" r:id="rId6"/>
+    <sheet name="ejemplo4_tabla_totales" sheetId="9" r:id="rId7"/>
+    <sheet name="ejemplo4_tabla_pagas" sheetId="10" r:id="rId8"/>
+    <sheet name="ejemplo5_tabla_sueldos_completo" sheetId="7" r:id="rId9"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">ejemplo4_tabla_pagas!#REF!</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">ejemplo4_tabla_sueldos!$A$1:$A$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">ejemplo4_tabla_totales!#REF!</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">MEDIANA!$A$1:$B$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Monstruo_Choco_Crunch!$B$1:$B$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">Oferta_Trabajo!$A$1:$B$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -46,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="65">
   <si>
     <t>Goles en la historia</t>
   </si>
@@ -196,14 +201,60 @@
   </si>
   <si>
     <t>retencion IRPF</t>
+  </si>
+  <si>
+    <t>Febrero</t>
+  </si>
+  <si>
+    <t>Marzo</t>
+  </si>
+  <si>
+    <t>Abril</t>
+  </si>
+  <si>
+    <t>Mayo</t>
+  </si>
+  <si>
+    <t>Julio</t>
+  </si>
+  <si>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>Septiembre</t>
+  </si>
+  <si>
+    <t>Octubre</t>
+  </si>
+  <si>
+    <t>Noviembre</t>
+  </si>
+  <si>
+    <t>Diciembre</t>
+  </si>
+  <si>
+    <t>Pagas</t>
+  </si>
+  <si>
+    <t>Mensualidad BRUTA</t>
+  </si>
+  <si>
+    <t>Mensualidad NETA</t>
+  </si>
+  <si>
+    <t>IRPF</t>
+  </si>
+  <si>
+    <t>SUELDO MEDIO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="#,##0\ &quot;€&quot;"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -246,7 +297,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -735,9 +786,6 @@
       <c r="B4">
         <v>2</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
@@ -872,16 +920,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="D3:F3"/>
+    <mergeCell ref="D5:F5"/>
+    <mergeCell ref="D7:F7"/>
+    <mergeCell ref="D9:F9"/>
+    <mergeCell ref="D10:F10"/>
     <mergeCell ref="D11:F11"/>
     <mergeCell ref="D13:F13"/>
     <mergeCell ref="D14:F14"/>
     <mergeCell ref="D15:F15"/>
     <mergeCell ref="D16:F16"/>
-    <mergeCell ref="D3:F3"/>
-    <mergeCell ref="D5:F5"/>
-    <mergeCell ref="D7:F7"/>
-    <mergeCell ref="D9:F9"/>
-    <mergeCell ref="D10:F10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1004,11 +1052,11 @@
   </sheetData>
   <autoFilter ref="A1:B8" xr:uid="{0BF25178-1294-4711-849D-35319D00EB7E}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B8">
-      <sortCondition ref="A9:A8"/>
+      <sortCondition ref="A8:A9"/>
     </sortState>
   </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B9">
-    <sortCondition ref="B10:B9"/>
+    <sortCondition ref="B9:B10"/>
   </sortState>
   <mergeCells count="4">
     <mergeCell ref="E6:G6"/>
@@ -1090,14 +1138,308 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA2105A3-0311-490E-A9E4-1EF0394880A4}">
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:D16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="25.5546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="35.5546875" customWidth="1"/>
+    <col min="1" max="1" width="35.5546875" customWidth="1"/>
+    <col min="2" max="2" width="25.5546875" style="2" customWidth="1"/>
+    <col min="3" max="3" width="35.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="7">
+        <v>18000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="7">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B3" s="7">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" s="7">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="7">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>45</v>
+      </c>
+      <c r="B6" s="7">
+        <v>60000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B7" s="7">
+        <v>89000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>47</v>
+      </c>
+      <c r="B8" s="7">
+        <v>300000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D12" s="1"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D14" s="2"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D15" s="2"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D16" s="2"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:A8" xr:uid="{DA2105A3-0311-490E-A9E4-1EF0394880A4}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FB56DC09-E9E8-468D-9F13-B8C6FEAA11D7}">
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="35.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="7">
+        <f>MEDIAN(ejemplo4_tabla_sueldos!B:B)</f>
+        <v>37500</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="7">
+        <f>AVERAGE(ejemplo4_tabla_sueldos!B:B)</f>
+        <v>74000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B3" s="1">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>60</v>
+      </c>
+      <c r="B4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="7">
+        <f>B1/B4</f>
+        <v>3125</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>63</v>
+      </c>
+      <c r="B6" s="7">
+        <f>B5*B3</f>
+        <v>562.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>62</v>
+      </c>
+      <c r="B7" s="7">
+        <f>B5-B6</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61DC0709-4017-458B-95EE-33940F44C4FE}">
+  <dimension ref="A1:B13"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="3" width="35.5546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>5</v>
+      </c>
+      <c r="B2" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>51</v>
+      </c>
+      <c r="B4" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B5" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B6" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>6</v>
+      </c>
+      <c r="B7" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>58</v>
+      </c>
+      <c r="B12" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>59</v>
+      </c>
+      <c r="B13" s="7">
+        <f>ejemplo4_tabla_totales!$B$7</f>
+        <v>2562.5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CAFC89B0-ADFC-4C8D-A5DB-D6F5D111FB2A}">
+  <dimension ref="A1:P26"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="2">
         <v>18000</v>
       </c>
@@ -1105,7 +1447,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>20000</v>
       </c>
@@ -1113,15 +1455,15 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
-        <v>21000</v>
+        <v>30000</v>
       </c>
       <c r="B3" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>28000</v>
       </c>
@@ -1129,7 +1471,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2">
         <v>35000</v>
       </c>
@@ -1137,7 +1479,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2">
         <v>60000</v>
       </c>
@@ -1145,7 +1487,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2">
         <v>89000</v>
       </c>
@@ -1153,7 +1495,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2">
         <v>300000</v>
       </c>
@@ -1161,41 +1503,446 @@
         <v>47</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
       <c r="B10" t="s">
         <v>30</v>
       </c>
-      <c r="C10" s="2">
+      <c r="E10" s="2">
         <f>MEDIAN(A:A)</f>
-        <v>31500</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+        <v>32500</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
       <c r="B11" t="s">
         <v>48</v>
       </c>
-      <c r="C11" s="2">
+      <c r="E11" s="2">
         <f>AVERAGE(A:A)</f>
-        <v>71375</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+        <v>71937.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
       <c r="B12" t="s">
         <v>49</v>
       </c>
-      <c r="C12" s="1">
+      <c r="E12" s="1">
         <v>0.18</v>
       </c>
     </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2"/>
+      <c r="B13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E13">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2"/>
+      <c r="B14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E14" s="2">
+        <f>E10/E13</f>
+        <v>2708.3333333333335</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
+      <c r="B15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15" s="2">
+        <f>E14*E12</f>
+        <v>487.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2"/>
+      <c r="B16" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" s="2">
+        <f>E14-E15</f>
+        <v>2220.8333333333335</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
+    </row>
+    <row r="18" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
+      <c r="C18" t="s">
+        <v>61</v>
+      </c>
+      <c r="D18" t="s">
+        <v>63</v>
+      </c>
+      <c r="E18" t="s">
+        <v>5</v>
+      </c>
+      <c r="F18" t="s">
+        <v>50</v>
+      </c>
+      <c r="G18" t="s">
+        <v>51</v>
+      </c>
+      <c r="H18" t="s">
+        <v>52</v>
+      </c>
+      <c r="I18" t="s">
+        <v>53</v>
+      </c>
+      <c r="J18" t="s">
+        <v>6</v>
+      </c>
+      <c r="K18" t="s">
+        <v>54</v>
+      </c>
+      <c r="L18" t="s">
+        <v>55</v>
+      </c>
+      <c r="M18" t="s">
+        <v>56</v>
+      </c>
+      <c r="N18" t="s">
+        <v>57</v>
+      </c>
+      <c r="O18" t="s">
+        <v>58</v>
+      </c>
+      <c r="P18" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>18000</v>
+      </c>
+      <c r="B19" t="s">
+        <v>40</v>
+      </c>
+      <c r="C19">
+        <f>A19/E13</f>
+        <v>1500</v>
+      </c>
+      <c r="D19">
+        <f>C19*E12</f>
+        <v>270</v>
+      </c>
+      <c r="E19">
+        <f>$C$19-$D$19</f>
+        <v>1230</v>
+      </c>
+      <c r="F19">
+        <f t="shared" ref="F19:P19" si="0">$C$19-$D$19</f>
+        <v>1230</v>
+      </c>
+      <c r="G19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="H19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="I19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="J19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="K19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="L19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="M19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="N19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="O19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+      <c r="P19">
+        <f t="shared" si="0"/>
+        <v>1230</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>20000</v>
+      </c>
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C20" s="2">
+        <f>A20/E13</f>
+        <v>1666.6666666666667</v>
+      </c>
+      <c r="D20">
+        <f>C20*E12</f>
+        <v>300</v>
+      </c>
+      <c r="E20" s="2">
+        <f>$C$20-$D$20</f>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="F20" s="2">
+        <f t="shared" ref="F20:P20" si="1">$C$20-$D$20</f>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="G20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="H20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="I20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="J20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="K20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="L20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="M20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="N20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="O20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+      <c r="P20" s="2">
+        <f t="shared" si="1"/>
+        <v>1366.6666666666667</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>21000</v>
+      </c>
+      <c r="B21" t="s">
+        <v>41</v>
+      </c>
+      <c r="C21">
+        <f>A21/E13</f>
+        <v>1750</v>
+      </c>
+      <c r="D21">
+        <f>C21*E12</f>
+        <v>315</v>
+      </c>
+      <c r="E21">
+        <f>$C$21-$D$21</f>
+        <v>1435</v>
+      </c>
+      <c r="F21">
+        <f t="shared" ref="F21:P21" si="2">$C$21-$D$21</f>
+        <v>1435</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="H21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="K21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="L21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="M21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="N21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="O21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+      <c r="P21">
+        <f t="shared" si="2"/>
+        <v>1435</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>28000</v>
+      </c>
+      <c r="B22" t="s">
+        <v>43</v>
+      </c>
+      <c r="C22" s="2">
+        <f>A22/E13</f>
+        <v>2333.3333333333335</v>
+      </c>
+      <c r="D22">
+        <f>C22*E12</f>
+        <v>420</v>
+      </c>
+      <c r="E22" s="2">
+        <f>$C$22-$D$22</f>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="F22" s="2">
+        <f t="shared" ref="F22:P22" si="3">$C$22-$D$22</f>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="G22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="H22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="I22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="J22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="K22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="L22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="M22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="N22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="O22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+      <c r="P22" s="2">
+        <f t="shared" si="3"/>
+        <v>1913.3333333333335</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>35000</v>
+      </c>
+      <c r="B23" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="2">
+        <f>A23/E13</f>
+        <v>2916.6666666666665</v>
+      </c>
+      <c r="D23">
+        <f>C23*E12</f>
+        <v>525</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>60000</v>
+      </c>
+      <c r="B24" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24">
+        <f>A24/E13</f>
+        <v>5000</v>
+      </c>
+      <c r="D24">
+        <f>C24*E12</f>
+        <v>900</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>89000</v>
+      </c>
+      <c r="B25" t="s">
+        <v>46</v>
+      </c>
+      <c r="C25" s="2">
+        <f>A25/E13</f>
+        <v>7416.666666666667</v>
+      </c>
+      <c r="D25">
+        <f>C25*E12</f>
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>300000</v>
+      </c>
+      <c r="B26" t="s">
+        <v>47</v>
+      </c>
+      <c r="C26">
+        <f>A26/E13</f>
+        <v>25000</v>
+      </c>
+      <c r="D26">
+        <f>C26*E12</f>
+        <v>4500</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B8" xr:uid="{DA2105A3-0311-490E-A9E4-1EF0394880A4}">
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B8">
-      <sortCondition ref="A1:A8"/>
-    </sortState>
-  </autoFilter>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A1:B10">
-    <sortCondition ref="A1:A10"/>
-  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>